<commit_message>
starting over with business analytics
</commit_message>
<xml_diff>
--- a/docs/marketing/keyword-research/JokerLabs_Keyword_to_Page_Workbook.xlsx
+++ b/docs/marketing/keyword-research/JokerLabs_Keyword_to_Page_Workbook.xlsx
@@ -22,6 +22,7 @@
     <sheet name="12_Decisions" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="13_Definitions" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="14_Sources" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="15_Page_Delivery" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00_Start'!$A$1:$E$13</definedName>
@@ -49,7 +50,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -67,6 +68,9 @@
     </font>
     <font>
       <color rgb="00333333"/>
+    </font>
+    <font>
+      <color rgb="00145DAD"/>
     </font>
   </fonts>
   <fills count="4">
@@ -99,7 +103,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -117,6 +121,12 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -276,7 +286,7 @@
 </file>
 
 <file path=xl/tables/table13.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="T12Decisions" displayName="T12Decisions" ref="A1:J36" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="13" name="T12Decisions" displayName="T12Decisions" ref="A1:J41" headerRowCount="1">
   <autoFilter ref="A1:J36"/>
   <tableColumns count="10">
     <tableColumn id="1" name="Date"/>
@@ -313,6 +323,27 @@
     <tableColumn id="2" name="URL / reference"/>
     <tableColumn id="3" name="Use"/>
     <tableColumn id="4" name="Reviewed date"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="T15PageDelivery" displayName="T15PageDelivery" ref="A1:L9" headerRowCount="1">
+  <autoFilter ref="A1:L8"/>
+  <tableColumns count="12">
+    <tableColumn id="1" name="Delivery ID"/>
+    <tableColumn id="2" name="Topic"/>
+    <tableColumn id="3" name="Spanish URL"/>
+    <tableColumn id="4" name="English URL"/>
+    <tableColumn id="5" name="Implementation date"/>
+    <tableColumn id="6" name="Source evidence"/>
+    <tableColumn id="7" name="Implementation checks"/>
+    <tableColumn id="8" name="Browser check"/>
+    <tableColumn id="9" name="Deploy/index status"/>
+    <tableColumn id="10" name="Keyword validation"/>
+    <tableColumn id="11" name="Owner"/>
+    <tableColumn id="12" name="Next action"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -856,7 +887,11 @@
           <t>Record account access and live deployment; no campaign required</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -879,7 +914,11 @@
           <t>Same reporting windows and network; separate countries</t>
         </is>
       </c>
-      <c r="D3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -902,7 +941,11 @@
           <t>Import measured observations with run ID and raw filename</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -925,7 +968,11 @@
           <t>Dated organic URLs and buyer-task review</t>
         </is>
       </c>
-      <c r="D5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -948,7 +995,11 @@
           <t>Trends settings and anonymized buyer language</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -971,7 +1022,11 @@
           <t>One destination per cluster/market; hypotheses reviewed</t>
         </is>
       </c>
-      <c r="D7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -991,13 +1046,17 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Reviewed brief with actual proof and claims scope</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr"/>
+          <t>7 topics / 14 detail pages implemented locally and verified; deployment and keyword research pending.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Not started</t>
+          <t>In progress</t>
         </is>
       </c>
     </row>
@@ -1017,7 +1076,11 @@
           <t>Record reporting windows and attribution limitations</t>
         </is>
       </c>
-      <c r="D9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
           <t>Not started</t>
@@ -3554,7 +3617,7 @@
     <outlinePr summaryBelow="1" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J36"/>
+  <dimension ref="A1:J41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -3621,29 +3684,101 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="58" customHeight="1">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
-      <c r="H2" s="2" t="n"/>
+    <row r="2" ht="80" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>BUILD_20261016_DETAIL_PAGES</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>User authorized seven source-based topics in ES/EN before keyword validation. Implemented locally; research statuses retained.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>DEL_SOFTWARE; DEL_AI; DEL_AUTOMATION; DEL_INTEGRATION; DEL_FX-CLOSING; DEL_FX-RATES; DEL_FX-REPORTS</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Service clusters used /es/services; operational guide URLs were proposals.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>See 15_Page_Delivery for fourteen implemented detail URLs; research exports and deployment remain.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>New pages only; old hub and anchors preserved. Reciprocal EN/ES canonicals/alternates; sitemap expanded.</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="I2" s="2" t="n"/>
-      <c r="J2" s="2" t="n"/>
-    </row>
-    <row r="3" ht="58" customHeight="1">
-      <c r="A3" s="2" t="n"/>
-      <c r="B3" s="2" t="n"/>
-      <c r="C3" s="2" t="n"/>
-      <c r="D3" s="2" t="n"/>
-      <c r="E3" s="2" t="n"/>
-      <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
-      <c r="H3" s="2" t="n"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Production build + 22 rendered SEO/link checks + desktop/mobile browser checks passed. Not deployed; research validation pending.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="105" customHeight="1">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>DEL_FX_PLANS</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Apply approved proposal to the existing product page in ES/EN; preserve prices and assisted trial terms.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>DEL_FX_PLANS; approved pricing proposal; rendered price checks</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Existing Currency Exchange product page; no new route needed.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>/es/currency-exchange#cx-plans and English counterpart; deployment and keyword validation remain pending.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>None: existing page canonicals retained; pricing uses a section anchor.</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="I3" s="2" t="n"/>
-      <c r="J3" s="2" t="n"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Core/Growth prices, activation and editable plan inquiry verified. 7-day initial trial; month-total extension with paid annual membership. No payment or live email sent.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="58" customHeight="1">
       <c r="A4" s="2" t="n"/>
@@ -4040,6 +4175,211 @@
       <c r="H36" s="2" t="n"/>
       <c r="I36" s="2" t="n"/>
       <c r="J36" s="2" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>SCOPE_FX_FINANCE_RELEASE</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Core y Growth incluirán reportería, contabilidad y finanzas al lanzamiento, sin cambio de precios. Compromiso comercial; entrega integral pendiente.</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Planes_y_Precios_JokerLabs_Currency_Exchange_v2_2026-10-16.md; decisión del propietario 2026-10-16</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Backend contable existente; experiencia completa y conciliación pendientes de validación.</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Completar UI, gastos/ajustes, exportaciones y conciliación/reproceso; validar cierre y estados antes de liberar.</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Ninguno; no se crea página nueva.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Alcance documentado; no acredita implementación, despliegue ni validación de mercado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>SCOPE_FX_ONBOARDING</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Activación incluye configuración, parametrización, capacitación, acompañamiento de primera operación/cierre y carga inicial acordada. Importe sin cambio.</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Aprobación del propietario; propuesta comercial; content/currency-exchange-plans.ts</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Servicios de implementación propuestos, pendientes de confirmación comercial.</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Publicar alcance aprobado en /es/currency-exchange#cx-plans y equivalente inglés. Acordar carga inicial y agenda antes de iniciar.</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Alcance incluido en tarjetas y propuesta; no acredita prestación del servicio ni despliegue.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>GROWTH_CUSTOM_QUOTE</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Growth pasa a cotización personalizada; Core conserva precios. Importes históricos de Growth solo como referencia interna.</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Instrucción propietario; content/currency-exchange-plans.ts</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>/es/currency-exchange#cx-plans y equivalente inglés; acordar capacidad y acompañamiento antes de cotizar.</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Web y propuesta alineadas; sin cambios a cobros ni catálogo del backend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>CORE_ANNUAL_VAT_PROMO</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Mostrar equivalente mensual aproximado y pago anual visible: Core 1.250.000 COP + IVA primer año. 7 días de prueba; compra anual extiende a un mes total incluyendo los 7 días.</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Confirmación propietario; content/currency-exchange-plans.ts; propuesta</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Revisar /es/currency-exchange#cx-plans y #cx-trial; Growth cotizado, implementación separada.</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Copy ES/EN actualizado; no se crea cobro mensual ni se modifica facturación del backend.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>CORE_PRICE_109900</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Core: 109.900 COP + IVA equivalente mensual; pago anual lanzamiento 1.318.800 COP + IVA; ahorro 181.200 COP antes de IVA frente a anual regular 1.500.000. Sustituye CORE_ANNUAL_VAT_PROMO en importes.</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Confirmación propietario: acomoda el valor en consecuencia; propuesta y contenido ES/EN</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Revisar oferta local; coordinar catálogo de cobro antes de aceptar pagos.</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Web y propuesta actualizadas; Growth cotizado, implementación y prueba sin cambios. Backend no modificado.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:J36"/>
@@ -4550,6 +4890,595 @@
   </sheetData>
   <autoFilter ref="A1:D11"/>
   <printOptions horizontalCentered="1"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="10" max="10"/>
+    <col width="38" customWidth="1" min="11" max="11"/>
+    <col width="38" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Delivery ID</t>
+        </is>
+      </c>
+      <c r="B1" s="7" t="inlineStr">
+        <is>
+          <t>Topic</t>
+        </is>
+      </c>
+      <c r="C1" s="7" t="inlineStr">
+        <is>
+          <t>Spanish URL</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>English URL</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>Implementation date</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>Source evidence</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>Implementation checks</t>
+        </is>
+      </c>
+      <c r="H1" s="7" t="inlineStr">
+        <is>
+          <t>Browser check</t>
+        </is>
+      </c>
+      <c r="I1" s="7" t="inlineStr">
+        <is>
+          <t>Deploy/index status</t>
+        </is>
+      </c>
+      <c r="J1" s="7" t="inlineStr">
+        <is>
+          <t>Keyword validation</t>
+        </is>
+      </c>
+      <c r="K1" s="7" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="L1" s="7" t="inlineStr">
+        <is>
+          <t>Next action</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="85" customHeight="1">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>DEL_SOFTWARE</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Desarrollo de software a medida para tu operación</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>/es/services/desarrollo-software</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>/services/custom-software</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>money-exchange-backend/app/services/fx.py; currency-exchange/AGENTS.md</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16: production build/TypeScript, Navbar ESLint and 23 rendered SEO/link/price checks passed. Current Core annual 1.318.800 COP + IVA; Growth custom quote.</t>
+        </is>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16 Chrome localhost: all 20 workbook pages HTTP 200, one H1 and substantive content; ES/EN menus at 1440/390px expose services, guides, pricing/trial anchors; Escape and no horizontal overflow verified.</t>
+        </is>
+      </c>
+      <c r="I2" s="8" t="inlineStr">
+        <is>
+          <t>Local HTTP verified; public deployment and Search Console indexing not verified</t>
+        </is>
+      </c>
+      <c r="J2" s="8" t="inlineStr">
+        <is>
+          <t>Unchanged; Keyword Planner/SERP evidence pending</t>
+        </is>
+      </c>
+      <c r="K2" s="8" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="L2" s="8" t="inlineStr">
+        <is>
+          <t>Validate demand/intent; deploy; Search Console inspect</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="85" customHeight="1">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>DEL_AI</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>Inteligencia artificial aplicada al trabajo de tu empresa</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>/es/services/inteligencia-artificial</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>/services/artificial-intelligence</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>jokerlabs-intelligence-agent 2/README.md; scripts/run_agent.py (internal code/design reference)</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16: production build/TypeScript, Navbar ESLint and 23 rendered SEO/link/price checks passed. Current Core annual 1.318.800 COP + IVA; Growth custom quote.</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16 Chrome localhost: all 20 workbook pages HTTP 200, one H1 and substantive content; ES/EN menus at 1440/390px expose services, guides, pricing/trial anchors; Escape and no horizontal overflow verified.</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Local HTTP verified; public deployment and Search Console indexing not verified</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>Unchanged; Keyword Planner/SERP evidence pending</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="L3" s="8" t="inlineStr">
+        <is>
+          <t>Validate demand/intent; deploy; Search Console inspect</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="85" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>DEL_AUTOMATION</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Automatización de procesos con controles claros</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>/es/services/automatizacion</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>/services/process-automation</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>jokerlabs-intelligence-agent 2/README.md; money-exchange-backend/docs/scheduler-contract.md</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16: production build/TypeScript, Navbar ESLint and 23 rendered SEO/link/price checks passed. Current Core annual 1.318.800 COP + IVA; Growth custom quote.</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16 Chrome localhost: all 20 workbook pages HTTP 200, one H1 and substantive content; ES/EN menus at 1440/390px expose services, guides, pricing/trial anchors; Escape and no horizontal overflow verified.</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>Local HTTP verified; public deployment and Search Console indexing not verified</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>Unchanged; Keyword Planner/SERP evidence pending</t>
+        </is>
+      </c>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="L4" s="8" t="inlineStr">
+        <is>
+          <t>Validate demand/intent; deploy; Search Console inspect</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="85" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>DEL_INTEGRATION</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Integración de sistemas para conectar tu operación</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>/es/services/integraciones</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>/services/system-integrations</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>money-exchange-backend/docs/integrations/wompi.md; docs/PROJECT-HANDOFF.md</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16: production build/TypeScript, Navbar ESLint and 23 rendered SEO/link/price checks passed. Current Core annual 1.318.800 COP + IVA; Growth custom quote.</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16 Chrome localhost: all 20 workbook pages HTTP 200, one H1 and substantive content; ES/EN menus at 1440/390px expose services, guides, pricing/trial anchors; Escape and no horizontal overflow verified.</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>Local HTTP verified; public deployment and Search Console indexing not verified</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>Unchanged; Keyword Planner/SERP evidence pending</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
+        <is>
+          <t>Validate demand/intent; deploy; Search Console inspect</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="85" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>DEL_FX-CLOSING</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Cómo revisar diferencias en el cierre de caja de una casa de cambio</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>/es/recursos/cierre-caja-casa-cambio</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>/resources/exchange-house-cash-closing</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>money-exchange-backend/app/services/fx.py (close_shift); ReconciliationResultModal.tsx</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16: production build/TypeScript, Navbar ESLint and 23 rendered SEO/link/price checks passed. Current Core annual 1.318.800 COP + IVA; Growth custom quote.</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16 Chrome localhost: all 20 workbook pages HTTP 200, one H1 and substantive content; ES/EN menus at 1440/390px expose services, guides, pricing/trial anchors; Escape and no horizontal overflow verified.</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Local HTTP verified; public deployment and Search Console indexing not verified</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>Unchanged; Keyword Planner/SERP evidence pending</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="L6" s="8" t="inlineStr">
+        <is>
+          <t>Validate demand/intent; deploy; Search Console inspect</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="85" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>DEL_FX-RATES</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Cómo revisar cambios de tasas en tu casa de cambio</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>/es/recursos/control-tasas-casa-cambio</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>/resources/exchange-house-rate-control</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>money-exchange-backend/app/services/fx.py (update_rates); CashReportView.tsx</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16: production build/TypeScript, Navbar ESLint and 23 rendered SEO/link/price checks passed. Current Core annual 1.318.800 COP + IVA; Growth custom quote.</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16 Chrome localhost: all 20 workbook pages HTTP 200, one H1 and substantive content; ES/EN menus at 1440/390px expose services, guides, pricing/trial anchors; Escape and no horizontal overflow verified.</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>Local HTTP verified; public deployment and Search Console indexing not verified</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>Unchanged; Keyword Planner/SERP evidence pending</t>
+        </is>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="L7" s="8" t="inlineStr">
+        <is>
+          <t>Validate demand/intent; deploy; Search Console inspect</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="85" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>DEL_FX-REPORTS</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>De las operaciones a los archivos de reportes de tu casa de cambio</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>/es/recursos/reportes-casas-cambio-colombia</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>/resources/colombian-exchange-house-reports</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="F8" s="8" t="inlineStr">
+        <is>
+          <t>money-exchange-backend/app/services/dian.py; app/services/uiaf.py</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16: production build/TypeScript, Navbar ESLint and 23 rendered SEO/link/price checks passed. Current Core annual 1.318.800 COP + IVA; Growth custom quote.</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16 Chrome localhost: all 20 workbook pages HTTP 200, one H1 and substantive content; ES/EN menus at 1440/390px expose services, guides, pricing/trial anchors; Escape and no horizontal overflow verified.</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>Local HTTP verified; public deployment and Search Console indexing not verified</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>Unchanged; Keyword Planner/SERP evidence pending</t>
+        </is>
+      </c>
+      <c r="K8" s="8" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="L8" s="8" t="inlineStr">
+        <is>
+          <t>Validate demand/intent; deploy; Search Console inspect</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="105" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>DEL_FX_PLANS</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Currency Exchange: planes, precios y prueba de 7 días</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>/es/currency-exchange#cx-plans</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>/currency-exchange#cx-plans</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="F9" s="8" t="inlineStr">
+        <is>
+          <t>docs/marketing/proposals/Planes_y_Precios_JokerLabs_Currency_Exchange_v2_2026-10-16.md; content/currency-exchange-plans.ts; docs/marketing-strategy.md</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16: production build/TypeScript, Navbar ESLint and 23 rendered SEO/link/price checks passed. Current Core annual 1.318.800 COP + IVA; Growth custom quote.</t>
+        </is>
+      </c>
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>2026-10-16 Chrome localhost: all 20 workbook pages HTTP 200, one H1 and substantive content; ES/EN menus at 1440/390px expose services, guides, pricing/trial anchors; Escape and no horizontal overflow verified.</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Local HTTP verified; public deployment and Search Console indexing not verified</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>Unchanged; Keyword Planner/SERP evidence pending</t>
+        </is>
+      </c>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="L9" s="8" t="inlineStr">
+        <is>
+          <t>Confirm launch validity and contractual dates before payment; deploy and inspect public page. No new page URL or backend pricing change.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <tableParts count="1">
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -4670,7 +5599,11 @@
       <c r="G2" s="2" t="inlineStr"/>
       <c r="H2" s="2" t="inlineStr"/>
       <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
           <t>Country service research</t>
@@ -4711,7 +5644,11 @@
       <c r="G3" s="2" t="inlineStr"/>
       <c r="H3" s="2" t="inlineStr"/>
       <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
           <t>Service research only</t>
@@ -4752,7 +5689,11 @@
       <c r="G4" s="2" t="inlineStr"/>
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
           <t>Service research only</t>
@@ -4793,7 +5734,11 @@
       <c r="G5" s="2" t="inlineStr"/>
       <c r="H5" s="2" t="inlineStr"/>
       <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
           <t>Overlaps Colombia - do not add national + Cali volume</t>
@@ -5005,7 +5950,7 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Implemented locally; verify live</t>
+          <t>Verified locally: HTTP 200 + content; production/index pending</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -5024,8 +5969,16 @@
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
-      <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> NAV_AUDIT_2026-10-16: Chrome HTTP 200, one H1 and content; ES/EN desktop/mobile navigation checked. Public access not verified.</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="58" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -5045,7 +5998,7 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Implemented locally; verify live</t>
+          <t>Verified locally: HTTP 200 + content; production/index pending</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -5064,8 +6017,16 @@
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr"/>
-      <c r="I3" s="2" t="inlineStr"/>
-      <c r="J3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> NAV_AUDIT_2026-10-16: Chrome HTTP 200, one H1 and content; ES/EN desktop/mobile navigation checked. Public access not verified.</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="58" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -5085,7 +6046,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Implemented locally; verify live</t>
+          <t>Verified locally: HTTP 200 + content; production/index pending</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -5104,8 +6065,16 @@
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>DEL_FX_PLANS: Core/Growth pricing, activation and 7-day trial/month-total extension applied locally in ES/EN; prices preserved. Build + 23 SEO/link/price checks passed; deployment/indexing pending. NAV_AUDIT_2026-10-16: Chrome HTTP 200, one H1 and content; ES/EN desktop/mobile navigation checked. Public access not verified.</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="58" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -5125,7 +6094,7 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Implemented locally; verify live</t>
+          <t>Verified locally: HTTP 200 + content; production/index pending</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -5144,8 +6113,16 @@
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
-      <c r="I5" s="2" t="inlineStr"/>
-      <c r="J5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> NAV_AUDIT_2026-10-16: Chrome HTTP 200, one H1 and content; ES/EN desktop/mobile navigation checked. Public access not verified.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="58" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -5165,7 +6142,7 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Implemented locally; verify live</t>
+          <t>Verified locally: HTTP 200 + content; production/index pending</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
@@ -5184,8 +6161,16 @@
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
-      <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> NAV_AUDIT_2026-10-16: Chrome HTTP 200, one H1 and content; ES/EN desktop/mobile navigation checked. Public access not verified.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="58" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -5205,7 +6190,7 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Implemented locally; verify live</t>
+          <t>Verified locally: HTTP 200 + content; production/index pending</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -5224,8 +6209,16 @@
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr"/>
-      <c r="I7" s="2" t="inlineStr"/>
-      <c r="J7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>DEL_FX_PLANS: Core/Growth pricing, activation and 7-day trial/month-total extension applied locally in ES/EN; prices preserved. Build + 23 SEO/link/price checks passed; deployment/indexing pending. NAV_AUDIT_2026-10-16: Chrome HTTP 200, one H1 and content; ES/EN desktop/mobile navigation checked. Public access not verified.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="58" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -5245,17 +6238,17 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Proposed - not built</t>
+          <t>Verified locally: HTTP 200 + content; production/index pending</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Custom software</t>
+          <t>Desarrollo de software a medida para tu operación</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Research before creating</t>
+          <t>Validate keywords; deploy; inspect live URL</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
@@ -5264,8 +6257,16 @@
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
-      <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>DEL_SOFTWARE; source-based content authorized 2026-10-16; not keyword-validated. NAV_AUDIT_2026-10-16: Chrome HTTP 200, one H1 and content; ES/EN desktop/mobile navigation checked. Public access not verified.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="58" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -5285,17 +6286,17 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Proposed - not built</t>
+          <t>Verified locally: HTTP 200 + content; production/index pending</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Applied AI</t>
+          <t>Inteligencia artificial aplicada al trabajo de tu empresa</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Research before creating</t>
+          <t>Validate keywords; deploy; inspect live URL</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
@@ -5304,8 +6305,16 @@
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr"/>
-      <c r="I9" s="2" t="inlineStr"/>
-      <c r="J9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>DEL_AI; source-based content authorized 2026-10-16; not keyword-validated. NAV_AUDIT_2026-10-16: Chrome HTTP 200, one H1 and content; ES/EN desktop/mobile navigation checked. Public access not verified.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="58" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -5325,17 +6334,17 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Proposed - not built</t>
+          <t>Verified locally: HTTP 200 + content; production/index pending</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Process automation</t>
+          <t>Automatización de procesos con controles claros</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Research before creating</t>
+          <t>Validate keywords; deploy; inspect live URL</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
@@ -5344,8 +6353,16 @@
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr"/>
-      <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>DEL_AUTOMATION; source-based content authorized 2026-10-16; not keyword-validated. NAV_AUDIT_2026-10-16: Chrome HTTP 200, one H1 and content; ES/EN desktop/mobile navigation checked. Public access not verified.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="58" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -5365,17 +6382,17 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Proposed - not built</t>
+          <t>Verified locally: HTTP 200 + content; production/index pending</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>System integrations</t>
+          <t>Integración de sistemas para conectar tu operación</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Research before creating</t>
+          <t>Validate keywords; deploy; inspect live URL</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
@@ -5384,8 +6401,16 @@
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr"/>
-      <c r="I11" s="2" t="inlineStr"/>
-      <c r="J11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>DEL_INTEGRATION; source-based content authorized 2026-10-16; not keyword-validated. NAV_AUDIT_2026-10-16: Chrome HTTP 200, one H1 and content; ES/EN desktop/mobile navigation checked. Public access not verified.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="58" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -5405,27 +6430,35 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Proposed - not built</t>
+          <t>Verified locally: HTTP 200 + content; production/index pending</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Cash closing guide</t>
+          <t>Cómo revisar diferencias en el cierre de caja de una casa de cambio</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Research before creating</t>
+          <t>Validate keywords; deploy; inspect live URL</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Colombia product</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
-      <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>DEL_FX-CLOSING; source-based content authorized 2026-10-16; not keyword-validated. NAV_AUDIT_2026-10-16: Chrome HTTP 200, one H1 and content; ES/EN desktop/mobile navigation checked. Public access not verified.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="58" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
@@ -5445,27 +6478,35 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Proposed - not built</t>
+          <t>Verified locally: HTTP 200 + content; production/index pending</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Rate review guide</t>
+          <t>Cómo revisar cambios de tasas en tu casa de cambio</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Research before creating</t>
+          <t>Validate keywords; deploy; inspect live URL</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Colombia product</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
-      <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>DEL_FX-RATES; source-based content authorized 2026-10-16; not keyword-validated. NAV_AUDIT_2026-10-16: Chrome HTTP 200, one H1 and content; ES/EN desktop/mobile navigation checked. Public access not verified.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="58" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -5485,111 +6526,371 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Proposed - not built</t>
+          <t>Verified locally: HTTP 200 + content; production/index pending</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Reporting preparation guide</t>
+          <t>De las operaciones a los archivos de reportes de tu casa de cambio</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Research before creating</t>
+          <t>Validate keywords; deploy; inspect live URL</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Colombia product</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr"/>
-      <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15" ht="58" customHeight="1">
-      <c r="A15" s="2" t="n"/>
-      <c r="B15" s="2" t="n"/>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
-      <c r="G15" s="2" t="n"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>DEL_FX-REPORTS; source-based content authorized 2026-10-16; not keyword-validated. NAV_AUDIT_2026-10-16: Chrome HTTP 200, one H1 and content; ES/EN desktop/mobile navigation checked. Public access not verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="80" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>en_software</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>/services/custom-software</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Verified locally: HTTP 200 + content; production/index pending</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Custom software built around your operation</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Validate keywords; deploy; inspect live URL</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>CO/PE/MX services</t>
+        </is>
+      </c>
       <c r="H15" s="2" t="n"/>
-      <c r="I15" s="2" t="n"/>
-      <c r="J15" s="2" t="n"/>
-    </row>
-    <row r="16" ht="58" customHeight="1">
-      <c r="A16" s="2" t="n"/>
-      <c r="B16" s="2" t="n"/>
-      <c r="C16" s="2" t="n"/>
-      <c r="D16" s="2" t="n"/>
-      <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
-      <c r="G16" s="2" t="n"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>DEL_SOFTWARE; source-based content authorized 2026-10-16; not keyword-validated. NAV_AUDIT_2026-10-16: Chrome HTTP 200, one H1 and content; ES/EN desktop/mobile navigation checked. Public access not verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="80" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>en_ai</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>/services/artificial-intelligence</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Verified locally: HTTP 200 + content; production/index pending</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Applied artificial intelligence for business workflows</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Validate keywords; deploy; inspect live URL</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>CO/PE/MX services</t>
+        </is>
+      </c>
       <c r="H16" s="2" t="n"/>
-      <c r="I16" s="2" t="n"/>
-      <c r="J16" s="2" t="n"/>
-    </row>
-    <row r="17" ht="58" customHeight="1">
-      <c r="A17" s="2" t="n"/>
-      <c r="B17" s="2" t="n"/>
-      <c r="C17" s="2" t="n"/>
-      <c r="D17" s="2" t="n"/>
-      <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="n"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>DEL_AI; source-based content authorized 2026-10-16; not keyword-validated. NAV_AUDIT_2026-10-16: Chrome HTTP 200, one H1 and content; ES/EN desktop/mobile navigation checked. Public access not verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="80" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>en_automation</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>/services/process-automation</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Verified locally: HTTP 200 + content; production/index pending</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Process automation with clear controls</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Validate keywords; deploy; inspect live URL</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>CO/PE/MX services</t>
+        </is>
+      </c>
       <c r="H17" s="2" t="n"/>
-      <c r="I17" s="2" t="n"/>
-      <c r="J17" s="2" t="n"/>
-    </row>
-    <row r="18" ht="58" customHeight="1">
-      <c r="A18" s="2" t="n"/>
-      <c r="B18" s="2" t="n"/>
-      <c r="C18" s="2" t="n"/>
-      <c r="D18" s="2" t="n"/>
-      <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
-      <c r="G18" s="2" t="n"/>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>DEL_AUTOMATION; source-based content authorized 2026-10-16; not keyword-validated. NAV_AUDIT_2026-10-16: Chrome HTTP 200, one H1 and content; ES/EN desktop/mobile navigation checked. Public access not verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="80" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>en_integration</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>/services/system-integrations</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Verified locally: HTTP 200 + content; production/index pending</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>System integrations that connect your operation</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Validate keywords; deploy; inspect live URL</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>CO/PE/MX services</t>
+        </is>
+      </c>
       <c r="H18" s="2" t="n"/>
-      <c r="I18" s="2" t="n"/>
-      <c r="J18" s="2" t="n"/>
-    </row>
-    <row r="19" ht="58" customHeight="1">
-      <c r="A19" s="2" t="n"/>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
-      <c r="G19" s="2" t="n"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>DEL_INTEGRATION; source-based content authorized 2026-10-16; not keyword-validated. NAV_AUDIT_2026-10-16: Chrome HTTP 200, one H1 and content; ES/EN desktop/mobile navigation checked. Public access not verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="80" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>en_fx-closing</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>/resources/exchange-house-cash-closing</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Verified locally: HTTP 200 + content; production/index pending</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>How to review exchange-house cash closing differences</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Validate keywords; deploy; inspect live URL</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Colombia product</t>
+        </is>
+      </c>
       <c r="H19" s="2" t="n"/>
-      <c r="I19" s="2" t="n"/>
-      <c r="J19" s="2" t="n"/>
-    </row>
-    <row r="20" ht="58" customHeight="1">
-      <c r="A20" s="2" t="n"/>
-      <c r="B20" s="2" t="n"/>
-      <c r="C20" s="2" t="n"/>
-      <c r="D20" s="2" t="n"/>
-      <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="n"/>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>DEL_FX-CLOSING; source-based content authorized 2026-10-16; not keyword-validated. NAV_AUDIT_2026-10-16: Chrome HTTP 200, one H1 and content; ES/EN desktop/mobile navigation checked. Public access not verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="80" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>en_fx-rates</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>/resources/exchange-house-rate-control</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Verified locally: HTTP 200 + content; production/index pending</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>How to review rate changes at your exchange house</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Validate keywords; deploy; inspect live URL</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Colombia product</t>
+        </is>
+      </c>
       <c r="H20" s="2" t="n"/>
-      <c r="I20" s="2" t="n"/>
-      <c r="J20" s="2" t="n"/>
-    </row>
-    <row r="21" ht="58" customHeight="1">
-      <c r="A21" s="2" t="n"/>
-      <c r="B21" s="2" t="n"/>
-      <c r="C21" s="2" t="n"/>
-      <c r="D21" s="2" t="n"/>
-      <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
-      <c r="G21" s="2" t="n"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>DEL_FX-RATES; source-based content authorized 2026-10-16; not keyword-validated. NAV_AUDIT_2026-10-16: Chrome HTTP 200, one H1 and content; ES/EN desktop/mobile navigation checked. Public access not verified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="80" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>en_fx-reports</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>/resources/colombian-exchange-house-reports</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Verified locally: HTTP 200 + content; production/index pending</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>From transactions to exchange-house reporting files</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Validate keywords; deploy; inspect live URL</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Colombia product</t>
+        </is>
+      </c>
       <c r="H21" s="2" t="n"/>
-      <c r="I21" s="2" t="n"/>
-      <c r="J21" s="2" t="n"/>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>DEL_FX-REPORTS; source-based content authorized 2026-10-16; not keyword-validated. NAV_AUDIT_2026-10-16: Chrome HTTP 200, one H1 and content; ES/EN desktop/mobile navigation checked. Public access not verified.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="58" customHeight="1">
       <c r="A22" s="2" t="n"/>
@@ -21305,7 +22606,11 @@
           <t>Company inquiry</t>
         </is>
       </c>
-      <c r="U2" s="2" t="inlineStr"/>
+      <c r="U2" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="V2" s="2" t="inlineStr"/>
       <c r="W2" s="2" t="inlineStr"/>
     </row>
@@ -21381,7 +22686,11 @@
           <t>Company inquiry</t>
         </is>
       </c>
-      <c r="U3" s="2" t="inlineStr"/>
+      <c r="U3" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="V3" s="2" t="inlineStr"/>
       <c r="W3" s="2" t="inlineStr"/>
     </row>
@@ -21457,7 +22766,11 @@
           <t>Company inquiry</t>
         </is>
       </c>
-      <c r="U4" s="2" t="inlineStr"/>
+      <c r="U4" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="V4" s="2" t="inlineStr"/>
       <c r="W4" s="2" t="inlineStr"/>
     </row>
@@ -21499,17 +22812,17 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>/es/services</t>
+          <t>/es/services/desarrollo-software</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>Existing local route</t>
+          <t>Implemented locally; deploy/index check pending</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Evaluate split</t>
+          <t>Implemented; keyword validation pending</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr"/>
@@ -21533,9 +22846,21 @@
           <t>Project inquiry</t>
         </is>
       </c>
-      <c r="U5" s="2" t="inlineStr"/>
-      <c r="V5" s="2" t="inlineStr"/>
-      <c r="W5" s="2" t="inlineStr"/>
+      <c r="U5" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="V5" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="W5" s="2" t="inlineStr">
+        <is>
+          <t>DEL_SOFTWARE: validate intent/demand, deploy and inspect live URL. Source evidence in 15_Page_Delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="58" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -21575,17 +22900,17 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>/es/services</t>
+          <t>/es/services/desarrollo-software</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>Existing local route</t>
+          <t>Implemented locally; deploy/index check pending</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Evaluate split</t>
+          <t>Implemented; keyword validation pending</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
@@ -21609,9 +22934,21 @@
           <t>Project inquiry</t>
         </is>
       </c>
-      <c r="U6" s="2" t="inlineStr"/>
-      <c r="V6" s="2" t="inlineStr"/>
-      <c r="W6" s="2" t="inlineStr"/>
+      <c r="U6" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="W6" s="2" t="inlineStr">
+        <is>
+          <t>DEL_SOFTWARE: validate intent/demand, deploy and inspect live URL. Source evidence in 15_Page_Delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="58" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -21651,17 +22988,17 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>/es/services</t>
+          <t>/es/services/desarrollo-software</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>Existing local route</t>
+          <t>Implemented locally; deploy/index check pending</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Evaluate split</t>
+          <t>Implemented; keyword validation pending</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr"/>
@@ -21685,9 +23022,21 @@
           <t>Project inquiry</t>
         </is>
       </c>
-      <c r="U7" s="2" t="inlineStr"/>
-      <c r="V7" s="2" t="inlineStr"/>
-      <c r="W7" s="2" t="inlineStr"/>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="W7" s="2" t="inlineStr">
+        <is>
+          <t>DEL_SOFTWARE: validate intent/demand, deploy and inspect live URL. Source evidence in 15_Page_Delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="58" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -21727,17 +23076,17 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>/es/services</t>
+          <t>/es/services/inteligencia-artificial</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>Existing local route</t>
+          <t>Implemented locally; deploy/index check pending</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Evaluate split</t>
+          <t>Implemented; keyword validation pending</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr"/>
@@ -21761,9 +23110,21 @@
           <t>Project inquiry</t>
         </is>
       </c>
-      <c r="U8" s="2" t="inlineStr"/>
-      <c r="V8" s="2" t="inlineStr"/>
-      <c r="W8" s="2" t="inlineStr"/>
+      <c r="U8" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="V8" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="W8" s="2" t="inlineStr">
+        <is>
+          <t>DEL_AI: validate intent/demand, deploy and inspect live URL. Source evidence in 15_Page_Delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="58" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -21803,17 +23164,17 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>/es/services</t>
+          <t>/es/services/inteligencia-artificial</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>Existing local route</t>
+          <t>Implemented locally; deploy/index check pending</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Evaluate split</t>
+          <t>Implemented; keyword validation pending</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -21837,9 +23198,21 @@
           <t>Project inquiry</t>
         </is>
       </c>
-      <c r="U9" s="2" t="inlineStr"/>
-      <c r="V9" s="2" t="inlineStr"/>
-      <c r="W9" s="2" t="inlineStr"/>
+      <c r="U9" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="V9" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="W9" s="2" t="inlineStr">
+        <is>
+          <t>DEL_AI: validate intent/demand, deploy and inspect live URL. Source evidence in 15_Page_Delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="58" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -21879,17 +23252,17 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>/es/services</t>
+          <t>/es/services/inteligencia-artificial</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>Existing local route</t>
+          <t>Implemented locally; deploy/index check pending</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>Evaluate split</t>
+          <t>Implemented; keyword validation pending</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr"/>
@@ -21913,9 +23286,21 @@
           <t>Project inquiry</t>
         </is>
       </c>
-      <c r="U10" s="2" t="inlineStr"/>
-      <c r="V10" s="2" t="inlineStr"/>
-      <c r="W10" s="2" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="inlineStr">
+        <is>
+          <t>DEL_AI: validate intent/demand, deploy and inspect live URL. Source evidence in 15_Page_Delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="58" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
@@ -21955,17 +23340,17 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>/es/services</t>
+          <t>/es/services/automatizacion</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>Existing local route</t>
+          <t>Implemented locally; deploy/index check pending</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Evaluate split</t>
+          <t>Implemented; keyword validation pending</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr"/>
@@ -21989,9 +23374,21 @@
           <t>Project inquiry</t>
         </is>
       </c>
-      <c r="U11" s="2" t="inlineStr"/>
-      <c r="V11" s="2" t="inlineStr"/>
-      <c r="W11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>DEL_AUTOMATION: validate intent/demand, deploy and inspect live URL. Source evidence in 15_Page_Delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="58" customHeight="1">
       <c r="A12" s="2" t="inlineStr">
@@ -22031,17 +23428,17 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>/es/services</t>
+          <t>/es/services/automatizacion</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>Existing local route</t>
+          <t>Implemented locally; deploy/index check pending</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>Evaluate split</t>
+          <t>Implemented; keyword validation pending</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr"/>
@@ -22065,9 +23462,21 @@
           <t>Project inquiry</t>
         </is>
       </c>
-      <c r="U12" s="2" t="inlineStr"/>
-      <c r="V12" s="2" t="inlineStr"/>
-      <c r="W12" s="2" t="inlineStr"/>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>DEL_AUTOMATION: validate intent/demand, deploy and inspect live URL. Source evidence in 15_Page_Delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="58" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
@@ -22107,17 +23516,17 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>/es/services</t>
+          <t>/es/services/automatizacion</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>Existing local route</t>
+          <t>Implemented locally; deploy/index check pending</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Evaluate split</t>
+          <t>Implemented; keyword validation pending</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr"/>
@@ -22141,9 +23550,21 @@
           <t>Project inquiry</t>
         </is>
       </c>
-      <c r="U13" s="2" t="inlineStr"/>
-      <c r="V13" s="2" t="inlineStr"/>
-      <c r="W13" s="2" t="inlineStr"/>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>DEL_AUTOMATION: validate intent/demand, deploy and inspect live URL. Source evidence in 15_Page_Delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="58" customHeight="1">
       <c r="A14" s="2" t="inlineStr">
@@ -22183,17 +23604,17 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>/es/services</t>
+          <t>/es/services/integraciones</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>Existing local route</t>
+          <t>Implemented locally; deploy/index check pending</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Evaluate split</t>
+          <t>Implemented; keyword validation pending</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr"/>
@@ -22217,9 +23638,21 @@
           <t>Project inquiry</t>
         </is>
       </c>
-      <c r="U14" s="2" t="inlineStr"/>
-      <c r="V14" s="2" t="inlineStr"/>
-      <c r="W14" s="2" t="inlineStr"/>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>DEL_INTEGRATION: validate intent/demand, deploy and inspect live URL. Source evidence in 15_Page_Delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="58" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
@@ -22259,17 +23692,17 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>/es/services</t>
+          <t>/es/services/integraciones</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>Existing local route</t>
+          <t>Implemented locally; deploy/index check pending</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Evaluate split</t>
+          <t>Implemented; keyword validation pending</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr"/>
@@ -22293,9 +23726,21 @@
           <t>Project inquiry</t>
         </is>
       </c>
-      <c r="U15" s="2" t="inlineStr"/>
-      <c r="V15" s="2" t="inlineStr"/>
-      <c r="W15" s="2" t="inlineStr"/>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>DEL_INTEGRATION: validate intent/demand, deploy and inspect live URL. Source evidence in 15_Page_Delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="58" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
@@ -22335,17 +23780,17 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>/es/services</t>
+          <t>/es/services/integraciones</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>Existing local route</t>
+          <t>Implemented locally; deploy/index check pending</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Evaluate split</t>
+          <t>Implemented; keyword validation pending</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr"/>
@@ -22369,9 +23814,21 @@
           <t>Project inquiry</t>
         </is>
       </c>
-      <c r="U16" s="2" t="inlineStr"/>
-      <c r="V16" s="2" t="inlineStr"/>
-      <c r="W16" s="2" t="inlineStr"/>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>DEL_INTEGRATION: validate intent/demand, deploy and inspect live URL. Source evidence in 15_Page_Delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="58" customHeight="1">
       <c r="A17" s="2" t="inlineStr">
@@ -22445,7 +23902,11 @@
           <t>Project inquiry</t>
         </is>
       </c>
-      <c r="U17" s="2" t="inlineStr"/>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="V17" s="2" t="inlineStr"/>
       <c r="W17" s="2" t="inlineStr"/>
     </row>
@@ -22521,7 +23982,11 @@
           <t>Project inquiry</t>
         </is>
       </c>
-      <c r="U18" s="2" t="inlineStr"/>
+      <c r="U18" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="V18" s="2" t="inlineStr"/>
       <c r="W18" s="2" t="inlineStr"/>
     </row>
@@ -22597,7 +24062,11 @@
           <t>Product demo</t>
         </is>
       </c>
-      <c r="U19" s="2" t="inlineStr"/>
+      <c r="U19" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="V19" s="2" t="inlineStr"/>
       <c r="W19" s="2" t="inlineStr"/>
     </row>
@@ -22644,12 +24113,12 @@
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Implemented locally; deploy/index check pending</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>Research new guide</t>
+          <t>Implemented; keyword validation pending</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr"/>
@@ -22673,9 +24142,21 @@
           <t>Product demo</t>
         </is>
       </c>
-      <c r="U20" s="2" t="inlineStr"/>
-      <c r="V20" s="2" t="inlineStr"/>
-      <c r="W20" s="2" t="inlineStr"/>
+      <c r="U20" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="V20" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="W20" s="2" t="inlineStr">
+        <is>
+          <t>DEL_FX-CLOSING: validate intent/demand, deploy and inspect live URL. Source evidence in 15_Page_Delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="58" customHeight="1">
       <c r="A21" s="2" t="inlineStr">
@@ -22720,12 +24201,12 @@
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>Proposed</t>
+          <t>Implemented locally; deploy/index check pending</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>Research new guide</t>
+          <t>Implemented; keyword validation pending</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr"/>
@@ -22749,9 +24230,21 @@
           <t>Product demo</t>
         </is>
       </c>
-      <c r="U21" s="2" t="inlineStr"/>
-      <c r="V21" s="2" t="inlineStr"/>
-      <c r="W21" s="2" t="inlineStr"/>
+      <c r="U21" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="V21" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="W21" s="2" t="inlineStr">
+        <is>
+          <t>DEL_FX-RATES: validate intent/demand, deploy and inspect live URL. Source evidence in 15_Page_Delivery.</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="58" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
@@ -22825,9 +24318,17 @@
           <t>Product demo</t>
         </is>
       </c>
-      <c r="U22" s="2" t="inlineStr"/>
+      <c r="U22" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="V22" s="2" t="inlineStr"/>
-      <c r="W22" s="2" t="inlineStr"/>
+      <c r="W22" s="2" t="inlineStr">
+        <is>
+          <t>Supporting guide implemented: /es/recursos/reportes-casas-cambio-colombia. Validate commercial vs informational intent before remapping.</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="58" customHeight="1">
       <c r="A23" s="2" t="n"/>
@@ -23711,7 +25212,11 @@
           <t>Closing difference; rate changes; receipt; read-only access</t>
         </is>
       </c>
-      <c r="J2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Operational benefits; daily cases; reporting; planned capabilities; Core/Growth comparison; activation and terms; assisted 7-day trial; month-total annual extension; guides; inquiry</t>
+        </is>
+      </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
           <t>/es/services; relevant future guides</t>
@@ -23719,19 +25224,23 @@
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Request a product demo</t>
+          <t>Request trial or editable Core/Growth annual-plan inquiry</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Colombia reporting; human review; no available AI/invoicing claim</t>
+          <t>Original COP rates and activation preserved. 4 users/branch; Core 1 branch, Growth up to 5. Activation timing and contract terms agreed before payment. No checkout or backend billing changes.</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr"/>
-      <c r="O2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>Research pending</t>
+          <t>Implemented locally: plans, prices and trial; keyword/deployment pending</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr"/>
@@ -23754,163 +25263,539 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Proposed - not built</t>
+          <t>Implemented locally; deploy/index check pending</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Business buying custom software</t>
+          <t>Business buyer evaluating the specific service</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Pending research</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr"/>
-      <c r="H3" s="2" t="inlineStr"/>
+          <t>Pending Keyword Planner + SERP exports; editorial hypothesis only</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>Desarrollo de software a medida para tu operación | JokerLabs</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Desarrollo de software a medida para tu operación</t>
+        </is>
+      </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>Use verified project scope and authorized examples</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr"/>
+          <t>Un registro que deja de viajar entre herramientas; money-exchange-backend/app/services/fx.py; currency-exchange/AGENTS.md</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Empieza por el proceso que necesitas resolver; Lo que aporta nuestra experiencia de producto; example; steps; FAQ; related pages; inquiry</t>
+        </is>
+      </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>/es/services; relevant product evidence</t>
+          <t>Services hub + sibling service pages</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>Request a project conversation</t>
+          <t>Hablemos de tu proyecto de software</t>
         </is>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Cali base; CO/PE/MX coverage; no foreign office claim</t>
+          <t>Con base en Cali, Colombia, atendemos proyectos para empresas en Colombia, Perú y México. Integraciones, migración de datos y soporte se definen por proyecto.</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr"/>
-      <c r="O3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>Research pending</t>
+          <t>Implemented locally; research/deployment pending</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr"/>
     </row>
-    <row r="4" ht="58" customHeight="1">
-      <c r="A4" s="2" t="n"/>
-      <c r="B4" s="2" t="n"/>
-      <c r="C4" s="2" t="n"/>
-      <c r="D4" s="2" t="n"/>
-      <c r="E4" s="2" t="n"/>
-      <c r="F4" s="2" t="n"/>
-      <c r="G4" s="2" t="n"/>
-      <c r="H4" s="2" t="n"/>
-      <c r="I4" s="2" t="n"/>
-      <c r="J4" s="2" t="n"/>
-      <c r="K4" s="2" t="n"/>
-      <c r="L4" s="2" t="n"/>
-      <c r="M4" s="2" t="n"/>
+    <row r="4" ht="80" customHeight="1">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>BRIEF_AI</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>AI_CO_ES;AI_PE_ES;AI_MX_ES</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>/es/services/inteligencia-artificial</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Implemented locally; deploy/index check pending</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Business buyer evaluating the specific service</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Pending Keyword Planner + SERP exports; editorial hypothesis only</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Inteligencia artificial aplicada al trabajo de tu empresa | JokerLabs</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Inteligencia artificial aplicada al trabajo de tu empresa</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Preparar una revisión semanal de información; jokerlabs-intelligence-agent 2/README.md; scripts/run_agent.py (internal code/design reference)</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>De una tarea repetida a un piloto evaluable; Un ejemplo de trabajo del laboratorio; example; steps; FAQ; related pages; inquiry</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Services hub + sibling service pages</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr">
+        <is>
+          <t>Evaluemos tu caso de IA</t>
+        </is>
+      </c>
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>Los modelos pueden producir errores. El proyecto define revisión humana, alcance de acceso y condiciones de proveedores antes de su uso operativo.</t>
+        </is>
+      </c>
       <c r="N4" s="2" t="n"/>
-      <c r="O4" s="2" t="n"/>
-      <c r="P4" s="2" t="n"/>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>Implemented locally; research/deployment pending</t>
+        </is>
+      </c>
       <c r="Q4" s="2" t="n"/>
     </row>
-    <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="2" t="n"/>
-      <c r="B5" s="2" t="n"/>
-      <c r="C5" s="2" t="n"/>
-      <c r="D5" s="2" t="n"/>
-      <c r="E5" s="2" t="n"/>
-      <c r="F5" s="2" t="n"/>
-      <c r="G5" s="2" t="n"/>
-      <c r="H5" s="2" t="n"/>
-      <c r="I5" s="2" t="n"/>
-      <c r="J5" s="2" t="n"/>
-      <c r="K5" s="2" t="n"/>
-      <c r="L5" s="2" t="n"/>
-      <c r="M5" s="2" t="n"/>
+    <row r="5" ht="80" customHeight="1">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>BRIEF_AUTOMATION</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>AUTOMATION_CO_ES;AUTOMATION_PE_ES;AUTOMATION_MX_ES</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>/es/services/automatizacion</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Implemented locally; deploy/index check pending</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Business buyer evaluating the specific service</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Pending Keyword Planner + SERP exports; editorial hypothesis only</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>Automatización de procesos con controles claros | JokerLabs</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Automatización de procesos con controles claros</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Un reporte que necesita llegar a revisión; jokerlabs-intelligence-agent 2/README.md; money-exchange-backend/docs/scheduler-contract.md</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Elegir qué automatizar primero; Diseñar el camino cuando algo falla; example; steps; FAQ; related pages; inquiry</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Services hub + sibling service pages</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>Revisemos tu proceso repetitivo</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>El alcance depende de las herramientas, sus permisos y las condiciones de sus proveedores. No se activa ningún envío ni tarea por solicitar información.</t>
+        </is>
+      </c>
       <c r="N5" s="2" t="n"/>
-      <c r="O5" s="2" t="n"/>
-      <c r="P5" s="2" t="n"/>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>Implemented locally; research/deployment pending</t>
+        </is>
+      </c>
       <c r="Q5" s="2" t="n"/>
     </row>
-    <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="2" t="n"/>
-      <c r="B6" s="2" t="n"/>
-      <c r="C6" s="2" t="n"/>
-      <c r="D6" s="2" t="n"/>
-      <c r="E6" s="2" t="n"/>
-      <c r="F6" s="2" t="n"/>
-      <c r="G6" s="2" t="n"/>
-      <c r="H6" s="2" t="n"/>
-      <c r="I6" s="2" t="n"/>
-      <c r="J6" s="2" t="n"/>
-      <c r="K6" s="2" t="n"/>
-      <c r="L6" s="2" t="n"/>
-      <c r="M6" s="2" t="n"/>
+    <row r="6" ht="80" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>BRIEF_INTEGRATION</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>INTEGRATION_CO_ES;INTEGRATION_PE_ES;INTEGRATION_MX_ES</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>/es/services/integraciones</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Implemented locally; deploy/index check pending</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Business buyer evaluating the specific service</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Pending Keyword Planner + SERP exports; editorial hypothesis only</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Integración de sistemas para conectar tu operación | JokerLabs</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Integración de sistemas para conectar tu operación</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>El pago aparece pendiente al regresar; money-exchange-backend/docs/integrations/wompi.md; docs/PROJECT-HANDOFF.md</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Conectar un proceso, no solo dos aplicaciones; Una referencia concreta: los pagos del producto; example; steps; FAQ; related pages; inquiry</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Services hub + sibling service pages</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Hablemos de tus sistemas</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Las aprobaciones del proveedor, costos externos y mantenimiento se acuerdan en la propuesta. No se prometen certificaciones ni acceso que todavía no esté disponible.</t>
+        </is>
+      </c>
       <c r="N6" s="2" t="n"/>
-      <c r="O6" s="2" t="n"/>
-      <c r="P6" s="2" t="n"/>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>Implemented locally; research/deployment pending</t>
+        </is>
+      </c>
       <c r="Q6" s="2" t="n"/>
     </row>
-    <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="2" t="n"/>
-      <c r="B7" s="2" t="n"/>
-      <c r="C7" s="2" t="n"/>
-      <c r="D7" s="2" t="n"/>
-      <c r="E7" s="2" t="n"/>
-      <c r="F7" s="2" t="n"/>
-      <c r="G7" s="2" t="n"/>
-      <c r="H7" s="2" t="n"/>
-      <c r="I7" s="2" t="n"/>
-      <c r="J7" s="2" t="n"/>
-      <c r="K7" s="2" t="n"/>
-      <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="n"/>
+    <row r="7" ht="80" customHeight="1">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>BRIEF_FX_CLOSING</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>FX-CASH_CO_ES</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>/es/recursos/cierre-caja-casa-cambio</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Implemented locally; deploy/index check pending</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Exchange-house operator/owner reviewing a workflow</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Pending Keyword Planner + SERP exports; editorial hypothesis only</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>Cómo revisar diferencias en el cierre de caja de una casa de cambio | JokerLabs</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Cómo revisar diferencias en el cierre de caja de una casa de cambio</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Ejemplo ilustrativo: faltan 10 USD; money-exchange-backend/app/services/fx.py (close_shift); ReconciliationResultModal.tsx</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Comparar lo esperado con lo contado; Investigar con los movimientos registrados; example; steps; FAQ; related pages; inquiry</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Currency Exchange + sibling operational guides</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Ver este cierre en una demo</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Guía del flujo del producto, sujeta a permisos y configuración. Los valores son ejemplos; no son datos de clientes ni un procedimiento contable o regulatorio obligatorio.</t>
+        </is>
+      </c>
       <c r="N7" s="2" t="n"/>
-      <c r="O7" s="2" t="n"/>
-      <c r="P7" s="2" t="n"/>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>Implemented locally; research/deployment pending</t>
+        </is>
+      </c>
       <c r="Q7" s="2" t="n"/>
     </row>
-    <row r="8" ht="58" customHeight="1">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
-      <c r="E8" s="2" t="n"/>
-      <c r="F8" s="2" t="n"/>
-      <c r="G8" s="2" t="n"/>
-      <c r="H8" s="2" t="n"/>
-      <c r="I8" s="2" t="n"/>
-      <c r="J8" s="2" t="n"/>
-      <c r="K8" s="2" t="n"/>
-      <c r="L8" s="2" t="n"/>
-      <c r="M8" s="2" t="n"/>
+    <row r="8" ht="80" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>BRIEF_FX_RATES</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>FX-RATES_CO_ES</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>/es/recursos/control-tasas-casa-cambio</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Implemented locally; deploy/index check pending</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Exchange-house operator/owner reviewing a workflow</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Pending Keyword Planner + SERP exports; editorial hypothesis only</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Cómo revisar cambios de tasas en tu casa de cambio | JokerLabs</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Cómo revisar cambios de tasas en tu casa de cambio</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Ejemplo ilustrativo: una tasa cambia a media jornada; money-exchange-backend/app/services/fx.py (update_rates); CashReportView.tsx</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Distinguir referencia y tasa de operación; Seguir el historial del cambio; example; steps; FAQ; related pages; inquiry</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Currency Exchange + sibling operational guides</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Revisar tasas e historial en una demo</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>Las cifras son ilustrativas. Esta guía explica la revisión operativa del producto; no recomienda tasas ni sustituye las políticas comerciales de tu empresa.</t>
+        </is>
+      </c>
       <c r="N8" s="2" t="n"/>
-      <c r="O8" s="2" t="n"/>
-      <c r="P8" s="2" t="n"/>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>Implemented locally; research/deployment pending</t>
+        </is>
+      </c>
       <c r="Q8" s="2" t="n"/>
     </row>
-    <row r="9" ht="58" customHeight="1">
-      <c r="A9" s="2" t="n"/>
-      <c r="B9" s="2" t="n"/>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="2" t="n"/>
-      <c r="E9" s="2" t="n"/>
-      <c r="F9" s="2" t="n"/>
-      <c r="G9" s="2" t="n"/>
-      <c r="H9" s="2" t="n"/>
-      <c r="I9" s="2" t="n"/>
-      <c r="J9" s="2" t="n"/>
-      <c r="K9" s="2" t="n"/>
-      <c r="L9" s="2" t="n"/>
-      <c r="M9" s="2" t="n"/>
+    <row r="9" ht="80" customHeight="1">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>BRIEF_FX_REPORTS</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>FX-REPORT_CO_ES</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>/es/recursos/reportes-casas-cambio-colombia</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Implemented locally; deploy/index check pending</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Exchange-house operator/owner reviewing a workflow</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Pending Keyword Planner + SERP exports; editorial hypothesis only</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>De las operaciones a los archivos de reportes de tu casa de cambio | JokerLabs</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>De las operaciones a los archivos de reportes de tu casa de cambio</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Ejemplo ilustrativo: compras y ventas no se mezclan; money-exchange-backend/app/services/dian.py; app/services/uiaf.py</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Qué archivos contempla el producto; Qué revisar antes de continuar; example; steps; FAQ; related pages; inquiry</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Currency Exchange + sibling operational guides</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Conocer el flujo de reportes en una demo</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Guía de capacidades del producto, no asesoría normativa. No define obligaciones, plazos ni umbrales. Confirma requisitos vigentes con el responsable competente y fuentes oficiales antes de presentar.</t>
+        </is>
+      </c>
       <c r="N9" s="2" t="n"/>
-      <c r="O9" s="2" t="n"/>
-      <c r="P9" s="2" t="n"/>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>Camilo</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>Implemented locally; research/deployment pending</t>
+        </is>
+      </c>
       <c r="Q9" s="2" t="n"/>
     </row>
     <row r="10" ht="58" customHeight="1">

</xml_diff>